<commit_message>
Budget Planner v1.2: navigation fix, delivery artifacts, listing assets
- Fixed Start Here navigation links for Google Sheets compatibility
  (replaced openpyxl hyperlinks with plain tab-name text)
- Created delivery/ folder with buyer-facing files (no version numbers)
- Generated quick-start guide (MD + HTML + PDF via fpdf2)
- Generated 5 listing images (Pillow mock spreadsheet previews)
- Created google-sheets-copy-link.txt, release-notes.txt
- Created delivery zip with all buyer-facing files
- Updated PRODUCT_CATALOG.csv status to Packaging
- Updated NOW.md, NEXT_ACTIONS.md, BUILD_CHECKLIST.md
- Created FORMULA_AUDIT_REPORT.md and NAVIGATION_QA_REPORT.md
</commit_message>
<xml_diff>
--- a/01-product-factory/02-products/budget-planner-expense-tracker/artifacts/budget-planner-expense-tracker-v1.1.xlsx
+++ b/01-product-factory/02-products/budget-planner-expense-tracker/artifacts/budget-planner-expense-tracker-v1.1.xlsx
@@ -25,7 +25,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="MM/DD/YYYY"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -80,6 +80,14 @@
       <b val="1"/>
       <color rgb="002F5496"/>
       <sz val="16"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="000563C1"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="7">
@@ -141,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -179,6 +187,15 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -763,7 +780,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B31"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -1007,12 +1024,69 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>QUICK NAVIGATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  &gt;&gt;  Monthly Budget</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  &gt;&gt;  Expense Tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  &gt;&gt;  Bills Tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  &gt;&gt;  Debt Tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  &gt;&gt;  Savings Tracker</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  &gt;&gt;  Dashboard</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A1:B1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A39" r:id="rId6"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1023,7 +1097,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1065,6 +1139,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="G1" s="34" t="inlineStr">
+        <is>
+          <t>&lt;&lt; Back to Start Here</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -1088,7 +1167,7 @@
         <v>4500</v>
       </c>
       <c r="D3" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A3,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A3,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E3" s="14">
@@ -1112,7 +1191,7 @@
         <v>800</v>
       </c>
       <c r="D4" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A4,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A4,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E4" s="14">
@@ -1136,7 +1215,7 @@
         <v>200</v>
       </c>
       <c r="D5" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A5,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A5,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E5" s="14">
@@ -1156,11 +1235,11 @@
         <f>SUM(C3:C5)</f>
         <v/>
       </c>
-      <c r="D6" s="16">
+      <c r="D6" s="35">
         <f>SUM(D3:D5)</f>
         <v/>
       </c>
-      <c r="E6" s="16">
+      <c r="E6" s="35">
         <f>C6-D6</f>
         <v/>
       </c>
@@ -1188,7 +1267,7 @@
         <v>1200</v>
       </c>
       <c r="D9" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A9,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A9,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E9" s="14">
@@ -1212,7 +1291,7 @@
         <v>200</v>
       </c>
       <c r="D10" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A10,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A10,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E10" s="14">
@@ -1236,7 +1315,7 @@
         <v>400</v>
       </c>
       <c r="D11" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A11,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A11,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E11" s="14">
@@ -1260,7 +1339,7 @@
         <v>150</v>
       </c>
       <c r="D12" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A12,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A12,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E12" s="14">
@@ -1284,7 +1363,7 @@
         <v>150</v>
       </c>
       <c r="D13" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A13,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A13,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E13" s="14">
@@ -1308,7 +1387,7 @@
         <v>100</v>
       </c>
       <c r="D14" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A14,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A14,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E14" s="14">
@@ -1332,7 +1411,7 @@
         <v>100</v>
       </c>
       <c r="D15" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A15,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A15,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E15" s="14">
@@ -1356,7 +1435,7 @@
         <v>150</v>
       </c>
       <c r="D16" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A16,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A16,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E16" s="14">
@@ -1380,7 +1459,7 @@
         <v>100</v>
       </c>
       <c r="D17" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A17,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A17,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E17" s="14">
@@ -1404,7 +1483,7 @@
         <v>50</v>
       </c>
       <c r="D18" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A18,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A18,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E18" s="14">
@@ -1428,7 +1507,7 @@
         <v>80</v>
       </c>
       <c r="D19" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A19,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A19,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E19" s="14">
@@ -1452,7 +1531,7 @@
         <v>200</v>
       </c>
       <c r="D20" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A20,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A20,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E20" s="14">
@@ -1476,7 +1555,7 @@
         <v>100</v>
       </c>
       <c r="D21" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A21,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A21,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E21" s="14">
@@ -1496,11 +1575,11 @@
         <f>SUM(C9:C21)</f>
         <v/>
       </c>
-      <c r="D22" s="16">
+      <c r="D22" s="35">
         <f>SUM(D9:D21)</f>
         <v/>
       </c>
-      <c r="E22" s="16">
+      <c r="E22" s="35">
         <f>C22-D22</f>
         <v/>
       </c>
@@ -1528,7 +1607,7 @@
         <v>500</v>
       </c>
       <c r="D25" s="14">
-        <f>SUMIF('Expense Tracker'!B:B,A25,'Expense Tracker'!G:G)</f>
+        <f>SUMIF('Expense Tracker'!C:C,A25,'Expense Tracker'!G:G)</f>
         <v/>
       </c>
       <c r="E25" s="14">
@@ -1548,11 +1627,11 @@
         <f>SUM(C25:C25)</f>
         <v/>
       </c>
-      <c r="D26" s="16">
+      <c r="D26" s="35">
         <f>SUM(D25:D25)</f>
         <v/>
       </c>
-      <c r="E26" s="16">
+      <c r="E26" s="35">
         <f>C26-D26</f>
         <v/>
       </c>
@@ -1574,7 +1653,16 @@
     <cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" dxfId="1">
       <formula>0</formula>
     </cfRule>
+    <cfRule type="cellIs" priority="4" operator="lessThan" dxfId="0">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="greaterThanOrEqual" dxfId="1">
+      <formula>0</formula>
+    </cfRule>
   </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G1" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1585,7 +1673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1639,6 +1727,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="I1" s="34" t="inlineStr">
+        <is>
+          <t>&lt;&lt; Back to Start Here</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="32" t="n">
@@ -2254,6 +2347,9 @@
       <formula1>"Planned,Unplanned"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="I1" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2264,7 +2360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2312,6 +2408,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="H1" s="34" t="inlineStr">
+        <is>
+          <t>&lt;&lt; Back to Start Here</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="19" t="inlineStr">
@@ -2493,6 +2594,12 @@
       <formula>$E2="Unpaid"</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1">
+      <formula>$E2="Paid"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>$E2="Unpaid"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="4" dxfId="1">
       <formula>$E2="Paid"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2504,6 +2611,9 @@
       <formula1>"Paid,Unpaid,Upcoming"</formula1>
     </dataValidation>
   </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2514,7 +2624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2562,6 +2672,11 @@
           <t>Payoff Progress %</t>
         </is>
       </c>
+      <c r="H1" s="34" t="inlineStr">
+        <is>
+          <t>&lt;&lt; Back to Start Here</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="19" t="inlineStr">
@@ -2642,6 +2757,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H1" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2652,7 +2770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2694,6 +2812,11 @@
           <t>Target Date</t>
         </is>
       </c>
+      <c r="G1" s="34" t="inlineStr">
+        <is>
+          <t>&lt;&lt; Back to Start Here</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="19" t="inlineStr">
@@ -2765,6 +2888,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G1" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2775,7 +2901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -2789,6 +2915,11 @@
           <t>Financial Dashboard</t>
         </is>
       </c>
+      <c r="D1" s="34" t="inlineStr">
+        <is>
+          <t>&lt;&lt; Back to Start Here</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
@@ -2796,9 +2927,14 @@
           <t>Total Income</t>
         </is>
       </c>
-      <c r="B3" s="28">
-        <f>SUMIF('Monthly Budget'!B:B,"Income",'Monthly Budget'!D:D)</f>
-        <v/>
+      <c r="B3" s="14">
+        <f>SUMIF('Monthly Budget'!B:B,"Income",'Monthly Budget'!C:C)</f>
+        <v/>
+      </c>
+      <c r="C3" s="39" t="inlineStr">
+        <is>
+          <t>All income from Salary, Freelance, Side Hustle (planned)</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -2807,9 +2943,14 @@
           <t>Total Expenses</t>
         </is>
       </c>
-      <c r="B5" s="28">
+      <c r="B5" s="14">
         <f>SUMIF('Monthly Budget'!B:B,"Expense",'Monthly Budget'!D:D)</f>
         <v/>
+      </c>
+      <c r="C5" s="39" t="inlineStr">
+        <is>
+          <t>All spending tracked in Expense Tracker</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -2818,9 +2959,14 @@
           <t>Net Savings</t>
         </is>
       </c>
-      <c r="B7" s="28">
+      <c r="B7" s="14">
         <f>B3-B5</f>
         <v/>
+      </c>
+      <c r="C7" s="39" t="inlineStr">
+        <is>
+          <t>Income minus Expenses</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -2829,9 +2975,14 @@
           <t>Savings Rate %</t>
         </is>
       </c>
-      <c r="B9" s="29">
+      <c r="B9" s="36">
         <f>IFERROR(B7/B3,0)</f>
         <v/>
+      </c>
+      <c r="C9" s="39" t="inlineStr">
+        <is>
+          <t>Net Savings ÷ Total Income</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -2840,9 +2991,14 @@
           <t>Bills Due</t>
         </is>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="37">
         <f>COUNTIF('Bills Tracker'!E:E,"Unpaid")</f>
         <v/>
+      </c>
+      <c r="C11" s="39" t="inlineStr">
+        <is>
+          <t>Unpaid bills requiring attention</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -2851,9 +3007,14 @@
           <t>Debt Remaining</t>
         </is>
       </c>
-      <c r="B13" s="28">
+      <c r="B13" s="14">
         <f>SUM('Debt Tracker'!C:C)</f>
         <v/>
+      </c>
+      <c r="C13" s="39" t="inlineStr">
+        <is>
+          <t>Total outstanding debt balance</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -2862,9 +3023,14 @@
           <t>Avg Savings Progress</t>
         </is>
       </c>
-      <c r="B15" s="29">
+      <c r="B15" s="36">
         <f>AVERAGE('Savings Tracker'!E:E)</f>
         <v/>
+      </c>
+      <c r="C15" s="39" t="inlineStr">
+        <is>
+          <t>Average % of savings targets achieved</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -3073,7 +3239,7 @@
           <t>Income</t>
         </is>
       </c>
-      <c r="B39" s="31">
+      <c r="B39" s="38">
         <f>B3</f>
         <v/>
       </c>
@@ -3084,7 +3250,7 @@
           <t>Expenses</t>
         </is>
       </c>
-      <c r="B40" s="31">
+      <c r="B40" s="38">
         <f>B4</f>
         <v/>
       </c>
@@ -3095,7 +3261,7 @@
           <t>Net Savings</t>
         </is>
       </c>
-      <c r="B41" s="31">
+      <c r="B41" s="38">
         <f>B5</f>
         <v/>
       </c>
@@ -3104,7 +3270,10 @@
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>